<commit_message>
Netherland Testcase Added with Changes
</commit_message>
<xml_diff>
--- a/Data/testDataNetherland1.xlsx
+++ b/Data/testDataNetherland1.xlsx
@@ -1,20 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21EE3DC1-B5EB-4947-B8CB-492972676859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="160">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -205,7 +219,7 @@
     <t>DefaultWeeklyHours</t>
   </si>
   <si>
-    <t>10698625</t>
+    <t>10698740</t>
   </si>
   <si>
     <t>Passed</t>
@@ -217,13 +231,13 @@
     <t>Mevr</t>
   </si>
   <si>
-    <t>Karson</t>
+    <t>Donna</t>
   </si>
   <si>
     <t>Test</t>
   </si>
   <si>
-    <t>Toy</t>
+    <t>Walter</t>
   </si>
   <si>
     <t>071 025 8087</t>
@@ -343,13 +357,16 @@
     <t>40</t>
   </si>
   <si>
+    <t>10698741</t>
+  </si>
+  <si>
     <t>701 Store Management (Vulam Syhohu (8701689))</t>
   </si>
   <si>
-    <t>Charlotte</t>
-  </si>
-  <si>
-    <t>Quitzon</t>
+    <t>Alyson</t>
+  </si>
+  <si>
+    <t>Kessler</t>
   </si>
   <si>
     <t>Full-time( FT. )</t>
@@ -358,7 +375,7 @@
     <t>New</t>
   </si>
   <si>
-    <t>Auto 83807558</t>
+    <t>Auto 68990934</t>
   </si>
   <si>
     <t>Store Manager</t>
@@ -373,6 +390,12 @@
     <t>NL Management</t>
   </si>
   <si>
+    <t>Breanne</t>
+  </si>
+  <si>
+    <t>Krajcik</t>
+  </si>
+  <si>
     <t>Defined contract end date (Determined)</t>
   </si>
   <si>
@@ -418,7 +441,7 @@
     <t>Netherlands Stockroom Operative</t>
   </si>
   <si>
-    <t xml:space="preserve">Stockroom Operative (21) </t>
+    <t>Stockroom Operative (21) </t>
   </si>
   <si>
     <t>Stockroom Operative</t>
@@ -490,82 +513,90 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="14"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="9" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF040C28"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF4A4A4A"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF4A4A4A"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FF4A4A4A"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -574,13 +605,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.1499984740745262"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -588,6 +619,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -611,33 +647,55 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin"/>
-      <top style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -648,28 +706,42 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -775,6 +847,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
@@ -1056,12 +1132,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BM31"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="58.1796875" customWidth="1"/>
-    <col min="4" max="4" width="27.08984375" customWidth="1"/>
+    <col min="4" max="4" width="59" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="20.08984375" customWidth="1"/>
     <col min="10" max="10" width="21.54296875" customWidth="1"/>
@@ -1077,6 +1153,7 @@
     <col min="32" max="32" width="21.453125" customWidth="1"/>
     <col min="33" max="33" width="31.6328125" customWidth="1"/>
     <col min="34" max="34" width="27.36328125" customWidth="1"/>
+    <col min="36" max="36" width="40.6328125" customWidth="1"/>
     <col min="37" max="37" width="22.54296875" customWidth="1"/>
     <col min="38" max="38" width="32.7265625" customWidth="1"/>
     <col min="42" max="42" width="23.36328125" customWidth="1"/>
@@ -1096,7 +1173,7 @@
     <col min="65" max="65" width="37.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="51" customHeight="1" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:65" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1293,7 +1370,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" ht="87.5" customHeight="1" spans="2:65" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:65" ht="87.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="12" t="s">
         <v>63</v>
       </c>
@@ -1325,8 +1402,8 @@
         <v>72</v>
       </c>
       <c r="L2" s="17">
-        <f t="shared" ref="L2:L16" si="0">TODAY()-31</f>
-        <v>45739</v>
+        <f t="shared" ref="L2:L16" ca="1" si="0">TODAY()-31</f>
+        <v>45744</v>
       </c>
       <c r="M2" s="18" t="s">
         <v>73</v>
@@ -1374,12 +1451,12 @@
         <v>84</v>
       </c>
       <c r="AB2" s="21">
-        <f t="shared" ref="AB2:AB16" si="1">AG2</f>
-        <v>45739</v>
+        <f t="shared" ref="AB2:AB16" ca="1" si="1">AG2</f>
+        <v>45744</v>
       </c>
       <c r="AC2" s="26">
-        <f t="shared" ref="AC2:AC16" si="2">AG2</f>
-        <v>45739</v>
+        <f t="shared" ref="AC2:AC16" ca="1" si="2">AG2</f>
+        <v>45744</v>
       </c>
       <c r="AD2" s="27" t="s">
         <v>85</v>
@@ -1391,8 +1468,8 @@
         <v>87</v>
       </c>
       <c r="AG2" s="29">
-        <f t="shared" ref="AG2:AG16" si="3">L2</f>
-        <v>45739</v>
+        <f t="shared" ref="AG2:AG16" ca="1" si="3">L2</f>
+        <v>45744</v>
       </c>
       <c r="AH2" s="21">
         <v>44986</v>
@@ -1446,7 +1523,7 @@
         <v>98</v>
       </c>
       <c r="AY2" s="35">
-        <v>645667205</v>
+        <v>645667230</v>
       </c>
       <c r="AZ2" t="s">
         <v>99</v>
@@ -1491,23 +1568,27 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" ht="14.5" customHeight="1" spans="2:65" x14ac:dyDescent="0.25">
-      <c r="B3" s="12"/>
-      <c r="C3" s="13"/>
+    <row r="3" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>64</v>
+      </c>
       <c r="D3" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E3" t="s">
         <v>66</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G3" t="s">
         <v>68</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I3" s="16" t="s">
         <v>70</v>
@@ -1519,8 +1600,8 @@
         <v>72</v>
       </c>
       <c r="L3" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M3" s="18" t="s">
         <v>73</v>
@@ -1562,18 +1643,18 @@
         <v>82</v>
       </c>
       <c r="Z3" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AA3" s="25" t="s">
         <v>84</v>
       </c>
       <c r="AB3" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC3" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD3" s="27" t="s">
         <v>85</v>
@@ -1585,26 +1666,26 @@
         <v>85</v>
       </c>
       <c r="AG3" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH3" s="24" t="s">
         <v>85</v>
       </c>
       <c r="AI3" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AJ3" s="16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AK3" s="30" t="s">
         <v>89</v>
       </c>
       <c r="AL3" s="31" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AM3" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AN3" s="18" t="s">
         <v>92</v>
@@ -1628,7 +1709,7 @@
         <v>95</v>
       </c>
       <c r="AU3" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AV3" s="37">
         <v>251</v>
@@ -1679,19 +1760,29 @@
         <v>106</v>
       </c>
       <c r="BL3" s="38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BM3" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="4" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C4" s="39"/>
+      <c r="D4" s="14" t="s">
+        <v>110</v>
+      </c>
       <c r="E4" t="s">
         <v>66</v>
       </c>
+      <c r="F4" t="s">
+        <v>120</v>
+      </c>
       <c r="G4" t="s">
         <v>68</v>
       </c>
+      <c r="H4" t="s">
+        <v>121</v>
+      </c>
       <c r="I4" s="16" t="s">
         <v>70</v>
       </c>
@@ -1702,8 +1793,8 @@
         <v>72</v>
       </c>
       <c r="L4" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M4" s="18" t="s">
         <v>73</v>
@@ -1742,7 +1833,7 @@
         <v>81</v>
       </c>
       <c r="Y4" s="23" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="24" t="s">
         <v>83</v>
@@ -1751,25 +1842,25 @@
         <v>84</v>
       </c>
       <c r="AB4" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC4" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD4" s="27" t="s">
         <v>85</v>
       </c>
       <c r="AE4" s="28" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="AF4" s="28" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="AG4" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH4" s="21">
         <v>44986</v>
@@ -1778,13 +1869,13 @@
         <v>88</v>
       </c>
       <c r="AJ4" s="16" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="AK4" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="AL4" s="31" t="s">
         <v>123</v>
-      </c>
-      <c r="AL4" s="31" t="s">
-        <v>120</v>
       </c>
       <c r="AM4" s="30" t="s">
         <v>91</v>
@@ -1805,14 +1896,14 @@
         <v>94</v>
       </c>
       <c r="AS4" s="33">
-        <f>TODAY()+365</f>
-        <v>46135</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46140</v>
       </c>
       <c r="AT4" s="16" t="s">
         <v>95</v>
       </c>
       <c r="AU4" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AV4" s="37">
         <v>251</v>
@@ -1823,8 +1914,8 @@
       <c r="AX4" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY4" s="35">
-        <v>645667207</v>
+      <c r="AY4" s="37">
+        <v>123456782</v>
       </c>
       <c r="AZ4" t="s">
         <v>99</v>
@@ -1863,13 +1954,16 @@
         <v>106</v>
       </c>
       <c r="BL4" s="38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BM4" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="5" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D5" s="14" t="s">
+        <v>110</v>
+      </c>
       <c r="E5" t="s">
         <v>66</v>
       </c>
@@ -1886,8 +1980,8 @@
         <v>72</v>
       </c>
       <c r="L5" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M5" s="18" t="s">
         <v>73</v>
@@ -1929,18 +2023,18 @@
         <v>82</v>
       </c>
       <c r="Z5" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AA5" s="25" t="s">
         <v>84</v>
       </c>
       <c r="AB5" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC5" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD5" s="27" t="s">
         <v>85</v>
@@ -1952,26 +2046,26 @@
         <v>85</v>
       </c>
       <c r="AG5" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH5" s="24" t="s">
         <v>85</v>
       </c>
       <c r="AI5" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AJ5" s="16" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="AK5" s="30" t="s">
         <v>89</v>
       </c>
       <c r="AL5" s="31" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AM5" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AN5" s="18" t="s">
         <v>92</v>
@@ -1995,7 +2089,7 @@
         <v>95</v>
       </c>
       <c r="AU5" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AV5" s="37">
         <v>251</v>
@@ -2006,8 +2100,8 @@
       <c r="AX5" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY5" s="35">
-        <v>645667208</v>
+      <c r="AY5" s="37">
+        <v>456789321</v>
       </c>
       <c r="AZ5" t="s">
         <v>99</v>
@@ -2046,13 +2140,16 @@
         <v>106</v>
       </c>
       <c r="BL5" s="38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BM5" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="6" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D6" s="14" t="s">
+        <v>110</v>
+      </c>
       <c r="E6" t="s">
         <v>66</v>
       </c>
@@ -2069,8 +2166,8 @@
         <v>72</v>
       </c>
       <c r="L6" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M6" s="18" t="s">
         <v>73</v>
@@ -2118,12 +2215,12 @@
         <v>84</v>
       </c>
       <c r="AB6" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC6" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD6" s="27" t="s">
         <v>85</v>
@@ -2135,8 +2232,8 @@
         <v>85</v>
       </c>
       <c r="AG6" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH6" s="21">
         <v>44986</v>
@@ -2145,13 +2242,13 @@
         <v>88</v>
       </c>
       <c r="AJ6" s="16" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="AK6" s="30" t="s">
         <v>89</v>
       </c>
       <c r="AL6" s="31" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AM6" s="30" t="s">
         <v>91</v>
@@ -2178,7 +2275,7 @@
         <v>95</v>
       </c>
       <c r="AU6" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AV6" s="37">
         <v>251</v>
@@ -2189,8 +2286,8 @@
       <c r="AX6" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY6" s="35">
-        <v>645667209</v>
+      <c r="AY6" s="37">
+        <v>234567896</v>
       </c>
       <c r="AZ6" t="s">
         <v>99</v>
@@ -2229,13 +2326,16 @@
         <v>106</v>
       </c>
       <c r="BL6" s="38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BM6" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="7" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D7" s="14" t="s">
+        <v>110</v>
+      </c>
       <c r="E7" t="s">
         <v>66</v>
       </c>
@@ -2252,8 +2352,8 @@
         <v>72</v>
       </c>
       <c r="L7" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M7" s="18" t="s">
         <v>73</v>
@@ -2292,21 +2392,21 @@
         <v>81</v>
       </c>
       <c r="Y7" s="23" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="Z7" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AA7" s="25" t="s">
         <v>84</v>
       </c>
       <c r="AB7" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC7" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD7" s="27" t="s">
         <v>85</v>
@@ -2318,8 +2418,8 @@
         <v>85</v>
       </c>
       <c r="AG7" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH7" s="21">
         <v>44987</v>
@@ -2328,16 +2428,16 @@
         <v>88</v>
       </c>
       <c r="AJ7" s="16" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="AK7" s="30" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="AL7" s="31" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="AM7" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AN7" s="18" t="s">
         <v>92</v>
@@ -2355,14 +2455,14 @@
         <v>94</v>
       </c>
       <c r="AS7" s="33">
-        <f>TODAY()+365</f>
-        <v>46135</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46140</v>
       </c>
       <c r="AT7" s="16" t="s">
         <v>95</v>
       </c>
       <c r="AU7" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AV7" s="37">
         <v>251</v>
@@ -2373,8 +2473,8 @@
       <c r="AX7" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY7" s="35">
-        <v>645667210</v>
+      <c r="AY7" s="37">
+        <v>345678902</v>
       </c>
       <c r="AZ7" t="s">
         <v>99</v>
@@ -2413,13 +2513,16 @@
         <v>106</v>
       </c>
       <c r="BL7" s="38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BM7" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="8" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D8" s="14" t="s">
+        <v>110</v>
+      </c>
       <c r="E8" t="s">
         <v>66</v>
       </c>
@@ -2436,8 +2539,8 @@
         <v>72</v>
       </c>
       <c r="L8" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M8" s="18" t="s">
         <v>73</v>
@@ -2476,21 +2579,21 @@
         <v>81</v>
       </c>
       <c r="Y8" s="23" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="Z8" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AA8" s="25" t="s">
         <v>84</v>
       </c>
       <c r="AB8" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC8" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD8" s="27" t="s">
         <v>85</v>
@@ -2502,8 +2605,8 @@
         <v>85</v>
       </c>
       <c r="AG8" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH8" s="21">
         <v>44988</v>
@@ -2512,16 +2615,16 @@
         <v>88</v>
       </c>
       <c r="AJ8" s="16" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="AK8" s="30" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="AL8" s="31" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="AM8" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AN8" s="18" t="s">
         <v>92</v>
@@ -2539,14 +2642,14 @@
         <v>94</v>
       </c>
       <c r="AS8" s="33">
-        <f>TODAY()+365</f>
-        <v>46135</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46140</v>
       </c>
       <c r="AT8" s="16" t="s">
         <v>95</v>
       </c>
       <c r="AU8" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AV8" s="37">
         <v>251</v>
@@ -2557,8 +2660,8 @@
       <c r="AX8" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY8" s="35">
-        <v>645667211</v>
+      <c r="AY8" s="37">
+        <v>567890124</v>
       </c>
       <c r="AZ8" t="s">
         <v>99</v>
@@ -2597,13 +2700,16 @@
         <v>106</v>
       </c>
       <c r="BL8" s="38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BM8" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="9" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D9" s="14" t="s">
+        <v>110</v>
+      </c>
       <c r="E9" t="s">
         <v>66</v>
       </c>
@@ -2620,8 +2726,8 @@
         <v>72</v>
       </c>
       <c r="L9" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M9" s="18" t="s">
         <v>73</v>
@@ -2669,12 +2775,12 @@
         <v>84</v>
       </c>
       <c r="AB9" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC9" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD9" s="27" t="s">
         <v>85</v>
@@ -2686,8 +2792,8 @@
         <v>85</v>
       </c>
       <c r="AG9" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH9" s="21">
         <v>44989</v>
@@ -2696,13 +2802,13 @@
         <v>88</v>
       </c>
       <c r="AJ9" s="16" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="AK9" s="30" t="s">
         <v>89</v>
       </c>
       <c r="AL9" s="31" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="AM9" s="30" t="s">
         <v>91</v>
@@ -2729,7 +2835,7 @@
         <v>95</v>
       </c>
       <c r="AU9" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AV9" s="37">
         <v>251</v>
@@ -2740,8 +2846,8 @@
       <c r="AX9" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY9" s="35">
-        <v>645667212</v>
+      <c r="AY9" s="37">
+        <v>678901245</v>
       </c>
       <c r="AZ9" t="s">
         <v>99</v>
@@ -2780,13 +2886,16 @@
         <v>106</v>
       </c>
       <c r="BL9" s="38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BM9" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="10" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D10" s="14" t="s">
+        <v>65</v>
+      </c>
       <c r="E10" t="s">
         <v>66</v>
       </c>
@@ -2803,8 +2912,8 @@
         <v>72</v>
       </c>
       <c r="L10" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M10" s="18" t="s">
         <v>73</v>
@@ -2846,18 +2955,18 @@
         <v>82</v>
       </c>
       <c r="Z10" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AA10" s="25" t="s">
         <v>84</v>
       </c>
       <c r="AB10" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC10" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD10" s="27" t="s">
         <v>85</v>
@@ -2869,8 +2978,8 @@
         <v>87</v>
       </c>
       <c r="AG10" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH10" s="21">
         <v>44990</v>
@@ -2888,7 +2997,7 @@
         <v>90</v>
       </c>
       <c r="AM10" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AN10" s="18" t="s">
         <v>92</v>
@@ -2923,8 +3032,8 @@
       <c r="AX10" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY10" s="35">
-        <v>645667213</v>
+      <c r="AY10" s="37">
+        <v>649012346</v>
       </c>
       <c r="AZ10" t="s">
         <v>99</v>
@@ -2969,7 +3078,10 @@
         <v>108</v>
       </c>
     </row>
-    <row r="11" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D11" s="14" t="s">
+        <v>65</v>
+      </c>
       <c r="E11" t="s">
         <v>66</v>
       </c>
@@ -2986,8 +3098,8 @@
         <v>72</v>
       </c>
       <c r="L11" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M11" s="18" t="s">
         <v>73</v>
@@ -3026,7 +3138,7 @@
         <v>81</v>
       </c>
       <c r="Y11" s="23" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="Z11" s="24" t="s">
         <v>83</v>
@@ -3035,25 +3147,25 @@
         <v>84</v>
       </c>
       <c r="AB11" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC11" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD11" s="27" t="s">
         <v>85</v>
       </c>
       <c r="AE11" s="28" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AF11" s="28" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="AG11" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH11" s="21">
         <v>44991</v>
@@ -3065,10 +3177,10 @@
         <v>85</v>
       </c>
       <c r="AK11" s="30" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="AL11" s="31" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="AM11" s="30" t="s">
         <v>91</v>
@@ -3089,8 +3201,8 @@
         <v>94</v>
       </c>
       <c r="AS11" s="33">
-        <f>TODAY()+365</f>
-        <v>46135</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46140</v>
       </c>
       <c r="AT11" s="16" t="s">
         <v>95</v>
@@ -3099,7 +3211,7 @@
         <v>96</v>
       </c>
       <c r="AV11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AW11" s="18" t="s">
         <v>73</v>
@@ -3107,8 +3219,8 @@
       <c r="AX11" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY11" s="35">
-        <v>645667214</v>
+      <c r="AY11" s="40">
+        <v>640123457</v>
       </c>
       <c r="AZ11" t="s">
         <v>99</v>
@@ -3153,7 +3265,10 @@
         <v>108</v>
       </c>
     </row>
-    <row r="12" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D12" s="14" t="s">
+        <v>65</v>
+      </c>
       <c r="E12" t="s">
         <v>66</v>
       </c>
@@ -3170,8 +3285,8 @@
         <v>72</v>
       </c>
       <c r="L12" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M12" s="18" t="s">
         <v>73</v>
@@ -3213,31 +3328,31 @@
         <v>82</v>
       </c>
       <c r="Z12" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AA12" s="25" t="s">
         <v>84</v>
       </c>
       <c r="AB12" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC12" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD12" s="27" t="s">
         <v>85</v>
       </c>
       <c r="AE12" s="28" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AF12" s="28" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="AG12" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH12" s="21">
         <v>44992</v>
@@ -3252,10 +3367,10 @@
         <v>89</v>
       </c>
       <c r="AL12" s="31" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="AM12" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AN12" s="18" t="s">
         <v>92</v>
@@ -3282,7 +3397,7 @@
         <v>96</v>
       </c>
       <c r="AV12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="AW12" s="18" t="s">
         <v>73</v>
@@ -3290,8 +3405,8 @@
       <c r="AX12" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY12" s="35">
-        <v>645667215</v>
+      <c r="AY12" s="37">
+        <v>645678902</v>
       </c>
       <c r="AZ12" t="s">
         <v>99</v>
@@ -3336,7 +3451,10 @@
         <v>108</v>
       </c>
     </row>
-    <row r="13" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D13" s="14" t="s">
+        <v>65</v>
+      </c>
       <c r="E13" t="s">
         <v>66</v>
       </c>
@@ -3353,8 +3471,8 @@
         <v>72</v>
       </c>
       <c r="L13" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M13" s="18" t="s">
         <v>73</v>
@@ -3402,25 +3520,25 @@
         <v>84</v>
       </c>
       <c r="AB13" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC13" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD13" s="27" t="s">
         <v>85</v>
       </c>
       <c r="AE13" s="28" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="AF13" s="28" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="AG13" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH13" s="21">
         <v>44993</v>
@@ -3435,7 +3553,7 @@
         <v>89</v>
       </c>
       <c r="AL13" s="31" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="AM13" s="30" t="s">
         <v>91</v>
@@ -3465,7 +3583,7 @@
         <v>96</v>
       </c>
       <c r="AV13" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="AW13" s="18" t="s">
         <v>73</v>
@@ -3473,8 +3591,8 @@
       <c r="AX13" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY13" s="35">
-        <v>645667216</v>
+      <c r="AY13" s="37">
+        <v>646789013</v>
       </c>
       <c r="AZ13" t="s">
         <v>99</v>
@@ -3519,7 +3637,10 @@
         <v>108</v>
       </c>
     </row>
-    <row r="14" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D14" s="14" t="s">
+        <v>65</v>
+      </c>
       <c r="E14" t="s">
         <v>66</v>
       </c>
@@ -3536,8 +3657,8 @@
         <v>72</v>
       </c>
       <c r="L14" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M14" s="18" t="s">
         <v>73</v>
@@ -3576,34 +3697,34 @@
         <v>81</v>
       </c>
       <c r="Y14" s="23" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="Z14" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AA14" s="25" t="s">
         <v>84</v>
       </c>
       <c r="AB14" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC14" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD14" s="27" t="s">
         <v>85</v>
       </c>
       <c r="AE14" s="28" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="AF14" s="28" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="AG14" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH14" s="21">
         <v>44994</v>
@@ -3615,13 +3736,13 @@
         <v>85</v>
       </c>
       <c r="AK14" s="30" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="AL14" s="31" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="AM14" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AN14" s="18" t="s">
         <v>92</v>
@@ -3639,8 +3760,8 @@
         <v>94</v>
       </c>
       <c r="AS14" s="33">
-        <f>TODAY()+365</f>
-        <v>46135</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46140</v>
       </c>
       <c r="AT14" s="16" t="s">
         <v>95</v>
@@ -3649,7 +3770,7 @@
         <v>96</v>
       </c>
       <c r="AV14" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="AW14" s="18" t="s">
         <v>73</v>
@@ -3657,8 +3778,8 @@
       <c r="AX14" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY14" s="35">
-        <v>645667217</v>
+      <c r="AY14" s="37">
+        <v>647890124</v>
       </c>
       <c r="AZ14" t="s">
         <v>99</v>
@@ -3703,7 +3824,10 @@
         <v>108</v>
       </c>
     </row>
-    <row r="15" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D15" s="14" t="s">
+        <v>65</v>
+      </c>
       <c r="E15" t="s">
         <v>66</v>
       </c>
@@ -3720,8 +3844,8 @@
         <v>72</v>
       </c>
       <c r="L15" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M15" s="18" t="s">
         <v>73</v>
@@ -3769,25 +3893,25 @@
         <v>84</v>
       </c>
       <c r="AB15" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC15" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD15" s="27" t="s">
         <v>85</v>
       </c>
       <c r="AE15" s="28" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="AF15" s="28" t="s">
         <v>85</v>
       </c>
       <c r="AG15" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH15" s="21">
         <v>44995</v>
@@ -3802,7 +3926,7 @@
         <v>89</v>
       </c>
       <c r="AL15" s="31" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="AM15" s="30" t="s">
         <v>91</v>
@@ -3832,7 +3956,7 @@
         <v>96</v>
       </c>
       <c r="AV15" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="AW15" s="18" t="s">
         <v>73</v>
@@ -3840,8 +3964,8 @@
       <c r="AX15" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY15" s="35">
-        <v>645667218</v>
+      <c r="AY15" s="37">
+        <v>648901235</v>
       </c>
       <c r="AZ15" t="s">
         <v>99</v>
@@ -3886,7 +4010,10 @@
         <v>108</v>
       </c>
     </row>
-    <row r="16" ht="14.5" customHeight="1" spans="5:65" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D16" s="14" t="s">
+        <v>65</v>
+      </c>
       <c r="E16" t="s">
         <v>66</v>
       </c>
@@ -3903,8 +4030,8 @@
         <v>72</v>
       </c>
       <c r="L16" s="17">
-        <f t="shared" si="0"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45744</v>
       </c>
       <c r="M16" s="18" t="s">
         <v>73</v>
@@ -3943,7 +4070,7 @@
         <v>81</v>
       </c>
       <c r="Y16" s="23" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="Z16" s="24" t="s">
         <v>83</v>
@@ -3952,25 +4079,25 @@
         <v>84</v>
       </c>
       <c r="AB16" s="21">
-        <f t="shared" si="1"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45744</v>
       </c>
       <c r="AC16" s="26">
-        <f t="shared" si="2"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45744</v>
       </c>
       <c r="AD16" s="27" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="AE16" s="28" t="s">
         <v>86</v>
       </c>
       <c r="AF16" s="28" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="AG16" s="29">
-        <f t="shared" si="3"/>
-        <v>45739</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45744</v>
       </c>
       <c r="AH16" s="21">
         <v>44996</v>
@@ -3982,7 +4109,7 @@
         <v>85</v>
       </c>
       <c r="AK16" s="30" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="AL16" s="31" t="s">
         <v>90</v>
@@ -4023,8 +4150,8 @@
       <c r="AX16" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="AY16" s="35">
-        <v>645667219</v>
+      <c r="AY16" s="37">
+        <v>649012346</v>
       </c>
       <c r="AZ16" t="s">
         <v>99</v>
@@ -4069,159 +4196,120 @@
         <v>108</v>
       </c>
     </row>
-    <row r="17" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
-      <c r="BM17" s="39" t="s">
-        <v>156</v>
+    <row r="17" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="BM17" s="41" t="s">
+        <v>159</v>
       </c>
     </row>
-    <row r="18" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
-      <c r="BM18" s="39" t="s">
-        <v>156</v>
+    <row r="18" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="BM18" s="41" t="s">
+        <v>159</v>
       </c>
     </row>
-    <row r="19" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
-      <c r="BM19" s="39" t="s">
-        <v>156</v>
+    <row r="19" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="BM19" s="41" t="s">
+        <v>159</v>
       </c>
     </row>
-    <row r="20" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
-      <c r="BM20" s="39" t="s">
-        <v>156</v>
+    <row r="20" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="BM20" s="41" t="s">
+        <v>159</v>
       </c>
     </row>
-    <row r="21" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
-      <c r="BM21" s="39" t="s">
-        <v>156</v>
+    <row r="21" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="BM21" s="41" t="s">
+        <v>159</v>
       </c>
     </row>
-    <row r="22" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
-      <c r="BM22" s="39" t="s">
-        <v>156</v>
+    <row r="22" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="BM22" s="41" t="s">
+        <v>159</v>
       </c>
     </row>
-    <row r="23" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
-      <c r="BM23" s="39" t="s">
-        <v>156</v>
+    <row r="23" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="BM23" s="41" t="s">
+        <v>159</v>
       </c>
     </row>
-    <row r="24" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
-      <c r="BM24" s="39" t="s">
-        <v>156</v>
+    <row r="24" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="BM24" s="41" t="s">
+        <v>159</v>
       </c>
     </row>
-    <row r="25" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
-      <c r="BM25" s="39" t="s">
-        <v>156</v>
+    <row r="25" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="BM25" s="41" t="s">
+        <v>159</v>
       </c>
     </row>
-    <row r="26" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
+    <row r="26" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="BM26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="27" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
+    <row r="27" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="BM27" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="28" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
+    <row r="28" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="BM28" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="29" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
+    <row r="29" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="BM29" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="30" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
+    <row r="30" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="BM30" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="31" ht="14.5" customHeight="1" spans="65:65" x14ac:dyDescent="0.25">
+    <row r="31" spans="65:65" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="BM31" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="19">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA10:AA16">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA10:AA16 V10:V16 S10:S16 K10:K16 BK10:BK16" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($E4)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA2:AA3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA2:AA3 V2:V3 S2:S3 K2:K3 BK2:BK3 AI2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>INDIRECT(#REF!)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA4:AA16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA4:AA16 V4:V16 S4:S16 K4:K16 BK4:BK16" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>INDIRECT($E4)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI10:AI16">
-      <formula1>INDIRECT($E4)</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI10:AI16" xr:uid="{00000000-0002-0000-0000-000003000000}">
+      <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2">
-      <formula1>INDIRECT(#REF!)</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI4" xr:uid="{00000000-0002-0000-0000-000005000000}">
+      <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI4">
-      <formula1>INDIRECT($E4)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI6:AI16">
-      <formula1>INDIRECT($E4)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK10:BK16">
-      <formula1>INDIRECT($E4)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2:BK3">
-      <formula1>INDIRECT(#REF!)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK4:BK16">
-      <formula1>INDIRECT($E4)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K10:K16">
-      <formula1>INDIRECT($E4)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K3">
-      <formula1>INDIRECT(#REF!)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4:K16">
-      <formula1>INDIRECT($E4)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S10:S16">
-      <formula1>INDIRECT($E4)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S3">
-      <formula1>INDIRECT(#REF!)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S4:S16">
-      <formula1>INDIRECT($E4)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V10:V16">
-      <formula1>INDIRECT($E4)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V3">
-      <formula1>INDIRECT(#REF!)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V4:V16">
-      <formula1>INDIRECT($E4)</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI6:AI16" xr:uid="{00000000-0002-0000-0000-000006000000}">
+      <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="U2" r:id="rId1"/>
-    <hyperlink ref="U3" r:id="rId2"/>
-    <hyperlink ref="U4" r:id="rId3"/>
-    <hyperlink ref="U5" r:id="rId4"/>
-    <hyperlink ref="U6" r:id="rId5"/>
-    <hyperlink ref="U7" r:id="rId6"/>
-    <hyperlink ref="U8" r:id="rId7"/>
-    <hyperlink ref="U9" r:id="rId8"/>
-    <hyperlink ref="U10" r:id="rId9"/>
-    <hyperlink ref="U11" r:id="rId10"/>
-    <hyperlink ref="U12" r:id="rId11"/>
-    <hyperlink ref="U13" r:id="rId12"/>
-    <hyperlink ref="U14" r:id="rId13"/>
-    <hyperlink ref="U15" r:id="rId14"/>
-    <hyperlink ref="U16" r:id="rId15"/>
+    <hyperlink ref="U2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="U3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="U4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="U5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="U6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="U7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="U8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="U9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="U10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="U11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="U12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="U13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="U14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="U15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="U16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>